<commit_message>
feat: add LicenseID support in Excel templates and update documentation
</commit_message>
<xml_diff>
--- a/examples/excel_template/basic/survey_import_basic_example.xlsx
+++ b/examples/excel_template/basic/survey_import_basic_example.xlsx
@@ -65675,7 +65675,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -65750,31 +65750,43 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>LicenseID</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>CC-BY-4.0</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Required by the schema. Pick an SPDX ID, or Proprietary/Other.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
         <is>
           <t>ShortName</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>mood</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Version_en</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="n">
-        <v>1</v>
-      </c>
-    </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Version_de</t>
+          <t>Version_en</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
@@ -65784,199 +65796,233 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>Version_de</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>Citation</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>PRISM Docs Team (2026). Daily Mood Check (tutorial example).</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>Construct_en</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>Momentary mood</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>Construct_de</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>Momentane Stimmung</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
+    <row r="11">
+      <c r="A11" t="inlineStr">
         <is>
           <t>Instructions_en</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>Think about today and answer each question.</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>Instructions_de</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>Denken Sie an den heutigen Tag und beantworten Sie jede Frage.</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>StudyDescription_en</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>Four-item daily mood check-in, used as a tutorial example.</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>StudyDescription_de</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>Vierteiliger taeglicher Stimmungscheck, als Tutorial-Beispiel.</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
+    <row r="15">
+      <c r="A15" t="inlineStr">
         <is>
           <t>Keywords</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>mood;tutorial;example</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
+    <row r="16">
+      <c r="A16" t="inlineStr">
         <is>
           <t>Authors</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>PRISM Docs Team</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>DOI</t>
         </is>
       </c>
-      <c r="B16" s="2" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="B17" s="2" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
         <is>
           <t>Respondent</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>self</t>
         </is>
       </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Who answers the items.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
         <is>
           <t>AdministrationMethod</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>digital</t>
+          <t>online</t>
         </is>
       </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>How this instrument is delivered — not a general 'digital' catch-all.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
         <is>
           <t>SoftwarePlatform</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>PRISM Tutorial</t>
+          <t>Other</t>
         </is>
       </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Use Other unless it's really LimeSurvey/PsychoPy/Pavlovia/paper.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
         <is>
           <t>SoftwareVersion</t>
         </is>
       </c>
-      <c r="B20" s="2" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>unspecified</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Required here because AdministrationMethod isn't paper. Avoid 'n/a'/'NA' — pandas reads those as blank.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
         <is>
           <t>I18nLanguages</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t>en;de</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>Add more tags like fr, es, it as needed.</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
+    <row r="23">
+      <c r="A23" t="inlineStr">
         <is>
           <t>I18nDefaultLanguage</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="B23" s="2" t="inlineStr">
         <is>
           <t>en</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
+    <row r="24">
+      <c r="A24" t="inlineStr">
         <is>
           <t>TranslationMethod</t>
         </is>
       </c>
-      <c r="B23" s="2" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>forward-backward</t>
         </is>
@@ -65984,12 +66030,21 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
-  <dataValidations count="2">
-    <dataValidation sqref="B17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Respondent" prompt="Select who responded." type="list">
-      <formula1>"self,parent,teacher,clinician,observer,other"</formula1>
+  <dataValidations count="5">
+    <dataValidation sqref="B4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="LicenseID" prompt="Required. Pick an SPDX-style license ID, or Proprietary/Other." type="list">
+      <formula1>"CC-BY-4.0,CC-BY-SA-4.0,CC-BY-ND-4.0,CC-BY-NC-4.0,CC-BY-NC-SA-4.0,CC-BY-NC-ND-4.0,MIT,Apache-2.0,GPL-3.0-only,GPL-3.0-or-later,LGPL-3.0-only,BSD-3-Clause,Unlicense,PDDL-1.0,CC0-1.0,Proprietary,Other"</formula1>
     </dataValidation>
-    <dataValidation sqref="B18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="AdministrationMethod" prompt="Select administration mode." type="list">
-      <formula1>"paper,digital,interview,phone,web,app,other"</formula1>
+    <dataValidation sqref="B18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Respondent" prompt="Select who responded." type="list">
+      <formula1>"self,clinician,parent,teacher,caregiver,other"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="AdministrationMethod" prompt="Select administration mode." type="list">
+      <formula1>"online,paper,interview,phone,mixed"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="SoftwarePlatform" prompt="Select the platform used to administer this survey." type="list">
+      <formula1>"LimeSurvey,PsychoPy,Pavlovia,Paper and Pencil,Other"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="TranslationMethod" prompt="Select how translations were produced." type="list">
+      <formula1>"forward-backward,committee,parallel,original,validated-translation"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -66002,7 +66057,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="2" max="2"/>
@@ -66187,12 +66242,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Respondent</t>
+          <t>LicenseID</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Dropdown values: self, parent, teacher, clinician, observer, other.</t>
+          <t>Required. Dropdown of SPDX-style license IDs; use Proprietary or Other if none fit.</t>
         </is>
       </c>
     </row>
@@ -66204,32 +66259,117 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>AdministrationMethod</t>
+          <t>Respondent</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Dropdown values: paper, digital, interview, phone, web, app, other.</t>
+          <t>Dropdown values: self, clinician, parent, teacher, caregiver, other.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>AdministrationMethod</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Dropdown values: online, paper, interview, phone, mixed. Not a general 'digital' catch-all — pick the closest match.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>SoftwarePlatform</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Dropdown values: LimeSurvey, PsychoPy, Pavlovia, Paper and Pencil, Other.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>SoftwareVersion</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Required unless SoftwarePlatform is Paper and Pencil or AdministrationMethod is paper.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>General</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>TranslationMethod</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Dropdown values: forward-backward, committee, parallel, original, validated-translation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>Items/General</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>Header row / non-Value cells</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>Locked (read-only) so column names and field labels can't be edited by accident. Dropdowns are suggestions, not hard limits — typing a custom value is still allowed.</t>
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Items</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ItemID uniqueness</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>PRISM does not check that ItemIDs are unique against other templates when importing here — only within this workbook. Use an instrument-specific prefix (mood01, not q01) to avoid silent collisions with other templates in your project.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>